<commit_message>
Update P&L with new fDespesas data
https://claude.ai/code/session_01Bb3ciycnMnk9Z7WYwsqMvC
</commit_message>
<xml_diff>
--- a/fDespesas.xlsx
+++ b/fDespesas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://safbotafogo-my.sharepoint.com/personal/pedro_arruda_safbfr_com_br/Documents/Área de Trabalho/dash-ticket/dash-ticket/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="471" documentId="8_{67AE05FE-6E1B-475B-A4F4-B6B330ED8DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17109036-1A4A-4F99-A6C0-37C27B1D62DE}"/>
+  <xr:revisionPtr revIDLastSave="540" documentId="8_{67AE05FE-6E1B-475B-A4F4-B6B330ED8DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E338217-13BF-44AE-A94D-D390C667198C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{EDFA135F-C4A3-4169-82D0-23AF6FF8D749}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha3" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha3!$A$1:$C$2238</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha3!$A$1:$C$2635</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5483" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5530" uniqueCount="138">
   <si>
     <t>3-staff</t>
   </si>
@@ -448,6 +448,12 @@
   <si>
     <t>2026.04.01-CAMBR2-9</t>
   </si>
+  <si>
+    <t>2026.04.09-CAMSU6-FG</t>
+  </si>
+  <si>
+    <t>2026.04.12-CAMBR2-11</t>
+  </si>
 </sst>
 </file>
 
@@ -499,7 +505,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -515,6 +521,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,7 +858,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5678EE0-CC9A-471A-9C23-3550D5ACF566}">
-  <dimension ref="A1:F2741"/>
+  <dimension ref="A1:F2765"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.90625" style="2" bestFit="1" customWidth="1"/>
@@ -28718,13 +28727,13 @@
     </row>
     <row r="2532" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2532" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2532" s="5">
-        <v>-9755</v>
+        <v>-2750</v>
       </c>
       <c r="C2532" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2533" spans="1:3" x14ac:dyDescent="0.35">
@@ -28732,175 +28741,175 @@
         <v>4</v>
       </c>
       <c r="B2533" s="5">
-        <v>-8688</v>
+        <v>-10210</v>
       </c>
       <c r="C2533" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2534" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2534" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2534" s="5">
-        <v>-27000</v>
+        <v>-3500</v>
       </c>
       <c r="C2534" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2535" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2535" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2535" s="5">
-        <v>-3800</v>
+        <v>-3119.5</v>
       </c>
       <c r="C2535" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2536" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2536" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2536" s="5">
-        <v>-3500</v>
+        <v>-2560</v>
       </c>
       <c r="C2536" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2537" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2537" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2537" s="5">
-        <v>-3010</v>
+        <v>-2101.1999999999998</v>
       </c>
       <c r="C2537" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2538" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2538" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B2538" s="5">
-        <v>-3119.5</v>
+        <v>-6800</v>
       </c>
       <c r="C2538" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2539" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2539" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2539" s="5">
-        <v>-15046.25</v>
+        <v>-7675</v>
       </c>
       <c r="C2539" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2540" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2540" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2540" s="5">
-        <v>-15180</v>
+        <v>-7634.2</v>
       </c>
       <c r="C2540" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2541" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2541" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2541" s="5">
-        <v>-1835.4</v>
+        <v>-9741.5</v>
       </c>
       <c r="C2541" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2542" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2542" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B2542" s="5">
-        <v>-5400</v>
+        <v>-16581</v>
       </c>
       <c r="C2542" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2543" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2543" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2543" s="5">
-        <v>-6604</v>
+        <v>-1790</v>
       </c>
       <c r="C2543" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2544" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2544" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2544" s="5">
-        <v>-2750</v>
+        <v>-3200</v>
       </c>
       <c r="C2544" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2545" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2545" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2545" s="5">
-        <v>-8620</v>
+        <v>-643</v>
       </c>
       <c r="C2545" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2546" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2546" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2546" s="5">
-        <v>-1790</v>
+        <v>-400</v>
       </c>
       <c r="C2546" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2547" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2547" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2547" s="5">
-        <v>-643</v>
+        <v>-8800</v>
       </c>
       <c r="C2547" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2548" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2548" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2548" s="5">
-        <v>-3200</v>
+        <v>-8010</v>
       </c>
       <c r="C2548" s="2" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2549" spans="1:3" x14ac:dyDescent="0.35">
@@ -28908,219 +28917,219 @@
         <v>4</v>
       </c>
       <c r="B2549" s="5">
-        <v>-8440</v>
+        <v>-31895</v>
       </c>
       <c r="C2549" s="2" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2550" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2550" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2550" s="5">
-        <v>-8805</v>
+        <v>-23649.200000000001</v>
       </c>
       <c r="C2550" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2551" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2551" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2551" s="5">
-        <v>-8688</v>
+        <v>-8000</v>
       </c>
       <c r="C2551" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2552" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2552" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2552" s="5">
-        <v>-27000</v>
+        <v>-3550</v>
       </c>
       <c r="C2552" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2553" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2553" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2553" s="5">
-        <v>-3800</v>
+        <v>-6782.5</v>
       </c>
       <c r="C2553" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2554" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2554" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B2554" s="5">
-        <v>-3500</v>
+        <v>-42249.5</v>
       </c>
       <c r="C2554" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2555" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2555" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2555" s="5">
-        <v>-2710</v>
+        <v>-27280</v>
       </c>
       <c r="C2555" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2556" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2556" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2556" s="5">
-        <v>-3119.5</v>
+        <v>-2632.8</v>
       </c>
       <c r="C2556" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2557" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2557" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B2557" s="5">
-        <v>-13101</v>
+        <v>-6800</v>
       </c>
       <c r="C2557" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2558" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2558" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2558" s="5">
-        <v>-11337.26</v>
+        <v>-400</v>
       </c>
       <c r="C2558" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2559" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2559" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2559" s="5">
-        <v>-1894.92</v>
+        <v>-10335</v>
       </c>
       <c r="C2559" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2560" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2560" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2560" s="5">
-        <v>-5400</v>
+        <v>-360</v>
       </c>
       <c r="C2560" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2561" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2561" s="2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B2561" s="5">
-        <v>-6604</v>
+        <v>-4000</v>
       </c>
       <c r="C2561" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2562" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2562" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2562" s="5">
-        <v>-2750</v>
+        <v>-7150</v>
       </c>
       <c r="C2562" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2563" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2563" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2563" s="5">
-        <v>-7634.2</v>
+        <v>-20616.8</v>
       </c>
       <c r="C2563" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2564" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2564" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2564" s="5">
-        <v>-1790</v>
+        <v>-2510</v>
       </c>
       <c r="C2564" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2565" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2565" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2565" s="5">
         <v>-643</v>
       </c>
       <c r="C2565" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2566" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2566" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2566" s="5">
         <v>-3200</v>
       </c>
       <c r="C2566" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2567" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2567" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2567" s="5">
-        <v>-5580</v>
+        <v>-12790</v>
       </c>
       <c r="C2567" s="2" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2568" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2568" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2568" s="5">
-        <v>-17010</v>
+        <v>-2632.8</v>
       </c>
       <c r="C2568" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2569" spans="1:3" x14ac:dyDescent="0.35">
@@ -29128,197 +29137,197 @@
         <v>4</v>
       </c>
       <c r="B2569" s="5">
-        <v>-12366.9</v>
+        <v>-17490</v>
       </c>
       <c r="C2569" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2570" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2570" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2570" s="5">
-        <v>-27000</v>
+        <v>-8000</v>
       </c>
       <c r="C2570" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2571" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2571" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2571" s="5">
-        <v>-3800</v>
+        <v>-1286</v>
       </c>
       <c r="C2571" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2572" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2572" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2572" s="5">
-        <v>-8000</v>
+        <v>-1500</v>
       </c>
       <c r="C2572" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2573" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2573" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2573" s="5">
-        <v>-3100</v>
+        <v>-8207</v>
       </c>
       <c r="C2573" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2574" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2574" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2574" s="5">
-        <v>-4137</v>
+        <v>-400</v>
       </c>
       <c r="C2574" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2575" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2575" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2575" s="5">
-        <v>-26311.5</v>
+        <v>-16809.8</v>
       </c>
       <c r="C2575" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2576" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2576" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2576" s="5">
-        <v>-7690</v>
+        <v>-3400</v>
       </c>
       <c r="C2576" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2577" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2577" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B2577" s="5">
-        <v>-2632.89</v>
+        <v>-28656</v>
       </c>
       <c r="C2577" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2578" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2578" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2578" s="5">
-        <v>-8300</v>
+        <v>-18260</v>
       </c>
       <c r="C2578" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2579" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2579" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B2579" s="5">
-        <v>-400</v>
+        <v>-6800</v>
       </c>
       <c r="C2579" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2580" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2580" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2580" s="5">
-        <v>-880</v>
+        <v>-11491</v>
       </c>
       <c r="C2580" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2581" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2581" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2581" s="5">
-        <v>-8911</v>
+        <v>-20171.599999999999</v>
       </c>
       <c r="C2581" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2582" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2582" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2582" s="5">
-        <v>-2400</v>
+        <v>-3200</v>
       </c>
       <c r="C2582" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2583" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2583" s="2" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B2583" s="5">
-        <v>-3850</v>
+        <v>-2400</v>
       </c>
       <c r="C2583" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2584" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2584" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2584" s="5">
-        <v>-11650</v>
+        <v>-4400</v>
       </c>
       <c r="C2584" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2585" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2585" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2585" s="5">
-        <v>-1790</v>
+        <v>-8950</v>
       </c>
       <c r="C2585" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2586" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2586" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2586" s="5">
-        <v>-643</v>
+        <v>-1790</v>
       </c>
       <c r="C2586" s="2" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2587" spans="1:3" x14ac:dyDescent="0.35">
@@ -29326,241 +29335,241 @@
         <v>4</v>
       </c>
       <c r="B2587" s="5">
-        <v>-3200</v>
+        <v>-11570</v>
       </c>
       <c r="C2587" s="2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2588" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2588" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2588" s="5">
-        <v>-17500</v>
+        <v>-6887.2</v>
       </c>
       <c r="C2588" s="2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2589" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2589" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2589" s="5">
-        <v>-7690</v>
+        <v>-6000</v>
       </c>
       <c r="C2589" s="2" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2590" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2590" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2590" s="5">
-        <v>-15410</v>
+        <v>-3100</v>
       </c>
       <c r="C2590" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2591" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2591" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2591" s="5">
-        <v>-19664.099999999999</v>
+        <v>-2509</v>
       </c>
       <c r="C2591" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2592" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2592" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B2592" s="5">
-        <v>-27000</v>
+        <v>-19002.5</v>
       </c>
       <c r="C2592" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2593" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2593" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2593" s="5">
-        <v>-3800</v>
+        <v>-14080</v>
       </c>
       <c r="C2593" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2594" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2594" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2594" s="5">
-        <v>-8000</v>
+        <v>-1569.6</v>
       </c>
       <c r="C2594" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2595" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2595" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B2595" s="5">
-        <v>-3700</v>
+        <v>-6800</v>
       </c>
       <c r="C2595" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2596" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2596" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2596" s="5">
-        <v>-7393</v>
+        <v>-400</v>
       </c>
       <c r="C2596" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2597" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2597" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2597" s="5">
-        <v>-31241.5</v>
+        <v>-8368</v>
       </c>
       <c r="C2597" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2598" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2598" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2598" s="5">
-        <v>-30688.79</v>
+        <v>-1925</v>
       </c>
       <c r="C2598" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2599" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2599" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2599" s="5">
-        <v>-2811.66</v>
+        <v>-11268.2</v>
       </c>
       <c r="C2599" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2600" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2600" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2600" s="5">
-        <v>-8300</v>
+        <v>-1790</v>
       </c>
       <c r="C2600" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2601" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2601" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2601" s="5">
-        <v>-400</v>
+        <v>-643</v>
       </c>
       <c r="C2601" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2602" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2602" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2602" s="5">
-        <v>-880</v>
+        <v>-3200</v>
       </c>
       <c r="C2602" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2603" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2603" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2603" s="5">
-        <v>-9775</v>
+        <v>-10010</v>
       </c>
       <c r="C2603" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2604" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2604" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2604" s="5">
-        <v>-4000</v>
+        <v>-8688</v>
       </c>
       <c r="C2604" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2605" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2605" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2605" s="5">
-        <v>-6600</v>
+        <v>-3500</v>
       </c>
       <c r="C2605" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2606" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2606" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2606" s="5">
-        <v>-14192</v>
+        <v>-3010</v>
       </c>
       <c r="C2606" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2607" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2607" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2607" s="5">
-        <v>-1790</v>
+        <v>-3119.5</v>
       </c>
       <c r="C2607" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2608" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2608" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B2608" s="5">
-        <v>-643</v>
+        <v>-15046.25</v>
       </c>
       <c r="C2608" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2609" spans="1:3" x14ac:dyDescent="0.35">
@@ -29568,175 +29577,175 @@
         <v>4</v>
       </c>
       <c r="B2609" s="5">
-        <v>-3051.2</v>
+        <v>-9755</v>
       </c>
       <c r="C2609" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2610" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2610" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2610" s="5">
-        <v>-17500</v>
+        <v>-15180</v>
       </c>
       <c r="C2610" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2611" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2611" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2611" s="5">
-        <v>-7510</v>
+        <v>-1835.4</v>
       </c>
       <c r="C2611" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2612" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2612" s="2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B2612" s="5">
-        <v>-1500</v>
+        <v>-5400</v>
       </c>
       <c r="C2612" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2613" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2613" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2613" s="5">
-        <v>-22670</v>
+        <v>-6604</v>
       </c>
       <c r="C2613" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2614" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2614" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2614" s="5">
-        <v>-23754.799999999999</v>
+        <v>-2750</v>
       </c>
       <c r="C2614" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2615" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2615" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2615" s="5">
-        <v>-27000</v>
+        <v>-8620</v>
       </c>
       <c r="C2615" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2616" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2616" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2616" s="5">
-        <v>-3800</v>
+        <v>-1790</v>
       </c>
       <c r="C2616" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2617" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2617" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2617" s="5">
-        <v>-12000</v>
+        <v>-643</v>
       </c>
       <c r="C2617" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2618" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2618" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2618" s="5">
-        <v>-4210</v>
+        <v>-3200</v>
       </c>
       <c r="C2618" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2619" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2619" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2619" s="5">
-        <v>-8207</v>
+        <v>-8440</v>
       </c>
       <c r="C2619" s="2" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2620" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2620" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2620" s="5">
-        <v>-53630.5</v>
-      </c>
-      <c r="C2620" s="2" t="s">
-        <v>120</v>
+        <v>-8688</v>
+      </c>
+      <c r="C2620" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2621" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2621" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2621" s="5">
-        <v>-41800</v>
-      </c>
-      <c r="C2621" s="2" t="s">
-        <v>120</v>
+        <v>-3500</v>
+      </c>
+      <c r="C2621" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2622" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2622" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2622" s="5">
-        <v>-4227.6899999999996</v>
-      </c>
-      <c r="C2622" s="2" t="s">
-        <v>120</v>
+        <v>-2710</v>
+      </c>
+      <c r="C2622" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2623" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2623" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2623" s="5">
-        <v>-8300</v>
-      </c>
-      <c r="C2623" s="2" t="s">
-        <v>120</v>
+        <v>-3119.5</v>
+      </c>
+      <c r="C2623" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2624" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2624" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B2624" s="5">
-        <v>-800</v>
-      </c>
-      <c r="C2624" s="2" t="s">
-        <v>120</v>
+        <v>-13101</v>
+      </c>
+      <c r="C2624" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2625" spans="1:3" x14ac:dyDescent="0.35">
@@ -29744,175 +29753,175 @@
         <v>4</v>
       </c>
       <c r="B2625" s="5">
-        <v>-10234</v>
-      </c>
-      <c r="C2625" s="2" t="s">
-        <v>120</v>
+        <v>-8805</v>
+      </c>
+      <c r="C2625" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2626" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2626" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2626" s="5">
-        <v>-6000</v>
-      </c>
-      <c r="C2626" s="2" t="s">
-        <v>120</v>
+        <v>-11337.26</v>
+      </c>
+      <c r="C2626" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2627" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2627" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2627" s="5">
-        <v>-7150</v>
-      </c>
-      <c r="C2627" s="2" t="s">
-        <v>120</v>
+        <v>-1894.92</v>
+      </c>
+      <c r="C2627" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2628" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2628" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B2628" s="5">
-        <v>-20491.400000000001</v>
-      </c>
-      <c r="C2628" s="2" t="s">
-        <v>120</v>
+        <v>-5400</v>
+      </c>
+      <c r="C2628" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2629" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2629" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2629" s="5">
-        <v>-1790</v>
-      </c>
-      <c r="C2629" s="2" t="s">
-        <v>120</v>
+        <v>-6604</v>
+      </c>
+      <c r="C2629" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2630" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2630" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2630" s="5">
-        <v>-1286</v>
-      </c>
-      <c r="C2630" s="2" t="s">
-        <v>120</v>
+        <v>-2750</v>
+      </c>
+      <c r="C2630" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2631" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2631" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2631" s="5">
-        <v>-3200</v>
-      </c>
-      <c r="C2631" s="2" t="s">
-        <v>120</v>
+        <v>-7634.2</v>
+      </c>
+      <c r="C2631" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2632" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2632" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2632" s="5">
-        <v>-16000</v>
-      </c>
-      <c r="C2632" s="2" t="s">
-        <v>120</v>
+        <v>-1790</v>
+      </c>
+      <c r="C2632" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2633" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2633" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2633" s="5">
-        <v>-26725</v>
-      </c>
-      <c r="C2633" s="2" t="s">
-        <v>133</v>
+        <v>-643</v>
+      </c>
+      <c r="C2633" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2634" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2634" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2634" s="5">
-        <v>-18977.400000000001</v>
-      </c>
-      <c r="C2634" s="2" t="s">
-        <v>133</v>
+        <v>-3200</v>
+      </c>
+      <c r="C2634" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2635" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2635" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2635" s="5">
-        <v>-27000</v>
-      </c>
-      <c r="C2635" s="2" t="s">
-        <v>133</v>
+        <v>-5580</v>
+      </c>
+      <c r="C2635" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="2636" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2636" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2636" s="5">
-        <v>-3800</v>
-      </c>
-      <c r="C2636" s="2" t="s">
-        <v>133</v>
+        <v>-12366.9</v>
+      </c>
+      <c r="C2636" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2637" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2637" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2637" s="5">
         <v>-8000</v>
       </c>
-      <c r="C2637" s="2" t="s">
-        <v>133</v>
+      <c r="C2637" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2638" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2638" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2638" s="5">
-        <v>-3550</v>
-      </c>
-      <c r="C2638" s="2" t="s">
-        <v>133</v>
+        <v>-3100</v>
+      </c>
+      <c r="C2638" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2639" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2639" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2639" s="5">
-        <v>-6172</v>
-      </c>
-      <c r="C2639" s="2" t="s">
-        <v>133</v>
+        <v>-4137</v>
+      </c>
+      <c r="C2639" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2640" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2640" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B2640" s="5">
-        <v>-40156.5</v>
-      </c>
-      <c r="C2640" s="2" t="s">
-        <v>133</v>
+        <v>-26311.5</v>
+      </c>
+      <c r="C2640" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2641" spans="1:3" x14ac:dyDescent="0.35">
@@ -29920,219 +29929,219 @@
         <v>4</v>
       </c>
       <c r="B2641" s="5">
-        <v>-27280</v>
-      </c>
-      <c r="C2641" s="2" t="s">
-        <v>133</v>
+        <v>-17010</v>
+      </c>
+      <c r="C2641" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2642" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2642" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2642" s="5">
-        <v>-2632.8</v>
-      </c>
-      <c r="C2642" s="2" t="s">
-        <v>133</v>
+        <v>-7690</v>
+      </c>
+      <c r="C2642" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2643" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2643" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2643" s="5">
-        <v>-6800</v>
-      </c>
-      <c r="C2643" s="2" t="s">
-        <v>133</v>
+        <v>-2632.89</v>
+      </c>
+      <c r="C2643" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2644" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2644" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B2644" s="5">
-        <v>-400</v>
-      </c>
-      <c r="C2644" s="2" t="s">
-        <v>133</v>
+        <v>-8300</v>
+      </c>
+      <c r="C2644" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2645" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2645" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2645" s="5">
-        <v>-9385</v>
-      </c>
-      <c r="C2645" s="2" t="s">
-        <v>133</v>
+        <v>-400</v>
+      </c>
+      <c r="C2645" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2646" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2646" s="2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B2646" s="5">
-        <v>-4000</v>
-      </c>
-      <c r="C2646" s="2" t="s">
-        <v>133</v>
+        <v>-880</v>
+      </c>
+      <c r="C2646" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2647" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2647" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2647" s="5">
-        <v>-5500</v>
-      </c>
-      <c r="C2647" s="2" t="s">
-        <v>133</v>
+        <v>-8911</v>
+      </c>
+      <c r="C2647" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2648" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2648" s="2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B2648" s="5">
-        <v>-12852.4</v>
-      </c>
-      <c r="C2648" s="2" t="s">
-        <v>133</v>
+        <v>-2400</v>
+      </c>
+      <c r="C2648" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2649" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2649" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2649" s="5">
-        <v>-2510</v>
-      </c>
-      <c r="C2649" s="2" t="s">
-        <v>133</v>
+        <v>-3850</v>
+      </c>
+      <c r="C2649" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2650" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2650" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2650" s="5">
-        <v>-964.5</v>
-      </c>
-      <c r="C2650" s="2" t="s">
-        <v>133</v>
+        <v>-11650</v>
+      </c>
+      <c r="C2650" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2651" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2651" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2651" s="5">
-        <v>-3200</v>
-      </c>
-      <c r="C2651" s="2" t="s">
-        <v>133</v>
+        <v>-1790</v>
+      </c>
+      <c r="C2651" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2652" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2652" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2652" s="5">
-        <v>-11530</v>
-      </c>
-      <c r="C2652" s="2" t="s">
-        <v>133</v>
+        <v>-643</v>
+      </c>
+      <c r="C2652" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2653" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2653" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2653" s="5">
-        <v>-6330</v>
-      </c>
-      <c r="C2653" s="2" t="s">
-        <v>132</v>
+        <v>-3200</v>
+      </c>
+      <c r="C2653" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2654" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2654" s="2" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B2654" s="5">
-        <v>-3500</v>
-      </c>
-      <c r="C2654" s="2" t="s">
-        <v>132</v>
+        <v>-17500</v>
+      </c>
+      <c r="C2654" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2655" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2655" s="2" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B2655" s="5">
-        <v>-2916</v>
-      </c>
-      <c r="C2655" s="2" t="s">
-        <v>132</v>
+        <v>-7690</v>
+      </c>
+      <c r="C2655" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="2656" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2656" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B2656" s="5">
-        <v>-27000</v>
+        <v>-19664.099999999999</v>
       </c>
       <c r="C2656" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2657" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2657" s="2" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B2657" s="5">
-        <v>-3800</v>
+        <v>-8000</v>
       </c>
       <c r="C2657" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2658" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2658" s="2" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="B2658" s="5">
-        <v>-2500</v>
+        <v>-3700</v>
       </c>
       <c r="C2658" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2659" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2659" s="2" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="B2659" s="5">
-        <v>-2367</v>
+        <v>-7393</v>
       </c>
       <c r="C2659" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2660" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2660" s="2" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="B2660" s="5">
-        <v>-4875</v>
+        <v>-31241.5</v>
       </c>
       <c r="C2660" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2661" spans="1:3" x14ac:dyDescent="0.35">
@@ -30140,208 +30149,208 @@
         <v>4</v>
       </c>
       <c r="B2661" s="5">
-        <v>-7540</v>
+        <v>-15410</v>
       </c>
       <c r="C2661" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2662" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2662" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2662" s="5">
-        <v>-7634.2</v>
+        <v>-30688.79</v>
       </c>
       <c r="C2662" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2663" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2663" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2663" s="5">
-        <v>-2750</v>
+        <v>-2811.66</v>
       </c>
       <c r="C2663" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2664" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2664" s="2" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B2664" s="5">
-        <v>-8688</v>
+        <v>-8300</v>
       </c>
       <c r="C2664" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2665" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2665" s="2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="B2665" s="5">
-        <v>-15479</v>
+        <v>-400</v>
       </c>
       <c r="C2665" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2666" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2666" s="2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B2666" s="5">
-        <v>-1790</v>
+        <v>-880</v>
       </c>
       <c r="C2666" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2667" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2667" s="2" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B2667" s="5">
-        <v>-3200</v>
+        <v>-9775</v>
       </c>
       <c r="C2667" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2668" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2668" s="2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B2668" s="5">
-        <v>-643</v>
+        <v>-4000</v>
       </c>
       <c r="C2668" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2669" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2669" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2669" s="5">
-        <v>-8010</v>
+        <v>-6600</v>
       </c>
       <c r="C2669" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2670" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2670" s="2" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="B2670" s="5">
-        <v>-2750</v>
+        <v>-14192</v>
       </c>
       <c r="C2670" s="2" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2671" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2671" s="2" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="B2671" s="5">
-        <v>-10210</v>
+        <v>-1790</v>
       </c>
       <c r="C2671" s="2" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2672" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2672" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B2672" s="5">
-        <v>-3500</v>
+        <v>-643</v>
       </c>
       <c r="C2672" s="2" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2673" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2673" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B2673" s="5">
-        <v>-3119.5</v>
+        <v>-3051.2</v>
       </c>
       <c r="C2673" s="2" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2674" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2674" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B2674" s="5">
-        <v>-2560</v>
+        <v>-17500</v>
       </c>
       <c r="C2674" s="2" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2675" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2675" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B2675" s="5">
-        <v>-2101.1999999999998</v>
+        <v>-7510</v>
       </c>
       <c r="C2675" s="2" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2676" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2676" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2676" s="5">
-        <v>-6800</v>
+        <v>-23754.799999999999</v>
       </c>
       <c r="C2676" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2677" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2677" s="2" t="s">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="B2677" s="5">
-        <v>-7675</v>
+        <v>-12000</v>
       </c>
       <c r="C2677" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2678" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2678" s="2" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B2678" s="5">
-        <v>-7634.2</v>
+        <v>-4210</v>
       </c>
       <c r="C2678" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2679" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2679" s="2" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B2679" s="5">
-        <v>-9741.5</v>
+        <v>-8207</v>
       </c>
       <c r="C2679" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2680" spans="1:3" x14ac:dyDescent="0.35">
@@ -30349,32 +30358,32 @@
         <v>0</v>
       </c>
       <c r="B2680" s="5">
-        <v>-16581</v>
+        <v>-53630.5</v>
       </c>
       <c r="C2680" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2681" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2681" s="2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="B2681" s="5">
-        <v>-1790</v>
+        <v>-22670</v>
       </c>
       <c r="C2681" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2682" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2682" s="2" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="B2682" s="5">
-        <v>-3200</v>
+        <v>-41800</v>
       </c>
       <c r="C2682" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2683" spans="1:3" x14ac:dyDescent="0.35">
@@ -30382,296 +30391,296 @@
         <v>19</v>
       </c>
       <c r="B2683" s="5">
-        <v>-643</v>
+        <v>-4227.6899999999996</v>
       </c>
       <c r="C2683" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2684" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2684" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B2684" s="5">
-        <v>-400</v>
+        <v>-8300</v>
       </c>
       <c r="C2684" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2685" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2685" s="2" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="B2685" s="5">
-        <v>-8800</v>
+        <v>-800</v>
       </c>
       <c r="C2685" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2686" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2686" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B2686" s="5">
-        <v>-8010</v>
+        <v>-10234</v>
       </c>
       <c r="C2686" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2687" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2687" s="2" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="B2687" s="5">
-        <v>-31895</v>
+        <v>-6000</v>
       </c>
       <c r="C2687" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2688" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2688" s="2" t="s">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="B2688" s="5">
-        <v>-23649.200000000001</v>
+        <v>-7150</v>
       </c>
       <c r="C2688" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2689" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2689" s="2" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B2689" s="5">
-        <v>-8000</v>
+        <v>-20491.400000000001</v>
       </c>
       <c r="C2689" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2690" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2690" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2690" s="5">
-        <v>-3550</v>
+        <v>-1790</v>
       </c>
       <c r="C2690" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2691" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2691" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B2691" s="5">
-        <v>-6782.5</v>
+        <v>-1286</v>
       </c>
       <c r="C2691" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2692" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2692" s="2" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="B2692" s="5">
-        <v>-42249.5</v>
+        <v>-3200</v>
       </c>
       <c r="C2692" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2693" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2693" s="2" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B2693" s="5">
-        <v>-27280</v>
+        <v>-16000</v>
       </c>
       <c r="C2693" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2694" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2694" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B2694" s="5">
-        <v>-2632.8</v>
+        <v>-1500</v>
       </c>
       <c r="C2694" s="2" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2695" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2695" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2695" s="5">
-        <v>-6800</v>
-      </c>
-      <c r="C2695" s="2" t="s">
-        <v>134</v>
+        <v>-18977.400000000001</v>
+      </c>
+      <c r="C2695" s="7" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="2696" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2696" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2696" s="5">
-        <v>-400</v>
+        <v>-8000</v>
       </c>
       <c r="C2696" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2697" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2697" s="2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B2697" s="5">
-        <v>-10335</v>
+        <v>-3550</v>
       </c>
       <c r="C2697" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2698" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2698" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B2698" s="5">
-        <v>-360</v>
+        <v>-6172</v>
       </c>
       <c r="C2698" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2699" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2699" s="2" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="B2699" s="5">
-        <v>-4000</v>
+        <v>-40156.5</v>
       </c>
       <c r="C2699" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2700" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2700" s="2" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="B2700" s="5">
-        <v>-7150</v>
+        <v>-26725</v>
       </c>
       <c r="C2700" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2701" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2701" s="2" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B2701" s="5">
-        <v>-20616.8</v>
+        <v>-27280</v>
       </c>
       <c r="C2701" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2702" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2702" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2702" s="5">
-        <v>-2510</v>
+        <v>-2632.8</v>
       </c>
       <c r="C2702" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2703" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2703" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B2703" s="5">
-        <v>-643</v>
+        <v>-6800</v>
       </c>
       <c r="C2703" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2704" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2704" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2704" s="5">
-        <v>-3200</v>
+        <v>-400</v>
       </c>
       <c r="C2704" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2705" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2705" s="2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B2705" s="5">
-        <v>-12790</v>
+        <v>-9385</v>
       </c>
       <c r="C2705" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2706" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2706" s="2" t="s">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="B2706" s="5">
-        <v>-2632.8</v>
+        <v>-4000</v>
       </c>
       <c r="C2706" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2707" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2707" s="2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="B2707" s="5">
-        <v>-17490</v>
+        <v>-5500</v>
       </c>
       <c r="C2707" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2708" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2708" s="2" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="B2708" s="5">
-        <v>-8000</v>
+        <v>-12852.4</v>
       </c>
       <c r="C2708" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2709" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2709" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B2709" s="5">
-        <v>-1286</v>
+        <v>-2510</v>
       </c>
       <c r="C2709" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2710" spans="1:3" x14ac:dyDescent="0.35">
@@ -30679,153 +30688,153 @@
         <v>19</v>
       </c>
       <c r="B2710" s="5">
-        <v>-1500</v>
+        <v>-964.5</v>
       </c>
       <c r="C2710" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2711" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2711" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B2711" s="5">
-        <v>-8207</v>
+        <v>-3200</v>
       </c>
       <c r="C2711" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2712" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2712" s="2" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="B2712" s="5">
-        <v>-400</v>
+        <v>-11530</v>
       </c>
       <c r="C2712" s="2" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2713" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2713" s="2" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="B2713" s="5">
-        <v>-16809.8</v>
+        <v>-3500</v>
       </c>
       <c r="C2713" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2714" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2714" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B2714" s="5">
-        <v>-3400</v>
+        <v>-2916</v>
       </c>
       <c r="C2714" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2715" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2715" s="2" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B2715" s="5">
-        <v>-28656</v>
+        <v>-6330</v>
       </c>
       <c r="C2715" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2716" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2716" s="2" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="B2716" s="5">
-        <v>-18260</v>
+        <v>-2500</v>
       </c>
       <c r="C2716" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2717" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2717" s="2" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B2717" s="5">
-        <v>-6800</v>
+        <v>-2367</v>
       </c>
       <c r="C2717" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2718" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2718" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B2718" s="5">
-        <v>-11491</v>
+        <v>-4875</v>
       </c>
       <c r="C2718" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2719" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2719" s="2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B2719" s="5">
-        <v>-20171.599999999999</v>
+        <v>-7540</v>
       </c>
       <c r="C2719" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2720" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2720" s="2" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="B2720" s="5">
-        <v>-3200</v>
+        <v>-7634.2</v>
       </c>
       <c r="C2720" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2721" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2721" s="2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B2721" s="5">
-        <v>-2400</v>
+        <v>-2750</v>
       </c>
       <c r="C2721" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2722" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2722" s="2" t="s">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="B2722" s="5">
-        <v>-4400</v>
+        <v>-8688</v>
       </c>
       <c r="C2722" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2723" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2723" s="2" t="s">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="B2723" s="5">
-        <v>-8950</v>
+        <v>-15479</v>
       </c>
       <c r="C2723" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2724" spans="1:3" x14ac:dyDescent="0.35">
@@ -30836,202 +30845,462 @@
         <v>-1790</v>
       </c>
       <c r="C2724" s="2" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2725" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2725" s="2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2725" s="5">
-        <v>-11570</v>
+        <v>-3200</v>
       </c>
       <c r="C2725" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2726" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2726" s="2" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="B2726" s="5">
-        <v>-6887.2</v>
+        <v>-643</v>
       </c>
       <c r="C2726" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2727" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2727" s="2" t="s">
-        <v>21</v>
+        <v>9</v>
       </c>
       <c r="B2727" s="5">
-        <v>-6000</v>
+        <v>-8010</v>
       </c>
       <c r="C2727" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="2728" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2728" s="2" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B2728" s="5">
-        <v>-3100</v>
+        <v>-11680.2</v>
       </c>
       <c r="C2728" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2729" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2729" s="2" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B2729" s="5">
-        <v>-2509</v>
+        <v>-6000</v>
       </c>
       <c r="C2729" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2730" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2730" s="2" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="B2730" s="5">
-        <v>-19002.5</v>
+        <v>-3010</v>
       </c>
       <c r="C2730" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2731" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2731" s="2" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="B2731" s="5">
-        <v>-14080</v>
+        <v>-4137</v>
       </c>
       <c r="C2731" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2732" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2732" s="2" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="B2732" s="5">
-        <v>-1569.6</v>
+        <v>-18882</v>
       </c>
       <c r="C2732" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2733" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2733" s="2" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B2733" s="5">
-        <v>-6800</v>
+        <v>-12420</v>
       </c>
       <c r="C2733" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2734" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2734" s="2" t="s">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="B2734" s="5">
-        <v>-400</v>
+        <v>-18260</v>
       </c>
       <c r="C2734" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2735" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2735" s="2" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B2735" s="5">
-        <v>-8368</v>
+        <v>-1835.8</v>
       </c>
       <c r="C2735" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2736" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2736" s="2" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="B2736" s="5">
-        <v>-1925</v>
+        <v>-6800</v>
       </c>
       <c r="C2736" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2737" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2737" s="2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B2737" s="5">
-        <v>-11268.2</v>
+        <v>-400</v>
       </c>
       <c r="C2737" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2738" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2738" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B2738" s="5">
-        <v>-1790</v>
+        <v>-200</v>
       </c>
       <c r="C2738" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2739" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2739" s="2" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B2739" s="5">
-        <v>-643</v>
+        <v>-9345</v>
       </c>
       <c r="C2739" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2740" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2740" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B2740" s="5">
-        <v>-3200</v>
+        <v>-3025</v>
       </c>
       <c r="C2740" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="2741" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2741" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2741" s="5">
+        <v>-12372.2</v>
+      </c>
+      <c r="C2741" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2742" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2742" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2742" s="5">
+        <v>-2510</v>
+      </c>
+      <c r="C2742" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2743" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2743" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2743" s="5">
+        <v>-1600</v>
+      </c>
+      <c r="C2743" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2744" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2744" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2744" s="5">
+        <v>-643</v>
+      </c>
+      <c r="C2744" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2745" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2745" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2745" s="5">
+        <v>-3200</v>
+      </c>
+      <c r="C2745" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2746" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2746" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2741" s="5">
-        <v>-10010</v>
-      </c>
-      <c r="C2741" s="2" t="s">
-        <v>135</v>
+      <c r="B2746" s="5">
+        <v>-13450</v>
+      </c>
+      <c r="C2746" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2747" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2747" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2747" s="5">
+        <v>-6306.1</v>
+      </c>
+      <c r="C2747" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2748" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2748" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2748" s="5">
+        <v>-8000</v>
+      </c>
+      <c r="C2748" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2749" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2749" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2749" s="5">
+        <v>-2500</v>
+      </c>
+      <c r="C2749" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2750" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2750" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2750" s="5">
+        <v>-3526.5</v>
+      </c>
+      <c r="C2750" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2751" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2751" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2751" s="5">
+        <v>-19781</v>
+      </c>
+      <c r="C2751" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2752" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2752" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2752" s="5">
+        <v>-12530</v>
+      </c>
+      <c r="C2752" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2753" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2753" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2753" s="5">
+        <v>-11220</v>
+      </c>
+      <c r="C2753" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2754" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2754" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2754" s="5">
+        <v>-1835.4</v>
+      </c>
+      <c r="C2754" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2755" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2755" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2755" s="5">
+        <v>-6800</v>
+      </c>
+      <c r="C2755" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2756" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2756" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2756" s="5">
+        <v>-200</v>
+      </c>
+      <c r="C2756" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2757" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2757" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2757" s="5">
+        <v>-8764</v>
+      </c>
+      <c r="C2757" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2758" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2758" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2758" s="5">
+        <v>-2200</v>
+      </c>
+      <c r="C2758" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2759" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2759" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2759" s="5">
+        <v>-11268.2</v>
+      </c>
+      <c r="C2759" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2760" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2760" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2760" s="5">
+        <v>-1790</v>
+      </c>
+      <c r="C2760" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2761" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2761" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2761" s="5">
+        <v>-800</v>
+      </c>
+      <c r="C2761" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2762" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2762" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2762" s="5">
+        <v>-400</v>
+      </c>
+      <c r="C2762" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2763" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2763" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2763" s="5">
+        <v>-643</v>
+      </c>
+      <c r="C2763" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2764" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2764" s="2" t="e">
+        <v>#N/A</v>
+      </c>
+      <c r="B2764" s="5">
+        <v>-3200</v>
+      </c>
+      <c r="C2764" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="2765" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2765" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2765" s="5">
+        <v>-10510</v>
+      </c>
+      <c r="C2765" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C2238" xr:uid="{E5678EE0-CC9A-471A-9C23-3550D5ACF566}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C2741">
-      <sortCondition ref="C1:C2238"/>
-    </sortState>
-  </autoFilter>
+  <autoFilter ref="A1:C2635" xr:uid="{E5678EE0-CC9A-471A-9C23-3550D5ACF566}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>